<commit_message>
Weeks 3 to 4 in the new mix (approved 30 Sep): 12 new posts, videos with music, LinkedIn PDFs, captions, schedule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW9n8unhL8LSAM1TzockVG
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule'!$A$1:$L$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule'!$A$1:$L$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4466,8 +4466,4268 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>15</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>P15A</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Nobody is coming to save your coaching business.</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>media/reels/p15a.mp4</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>captions/p15a.txt</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>15</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>P15B</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>4 leaks on this coach's page in 5 minutes.</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>media/v2/d15a/d15a.pdf</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>captions/d15a.txt</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>15</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>P15A</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Nobody is coming to save your coaching business.</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>media/reels/p15a.mp4</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>captions/p15a.txt</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>15</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>P15B</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>4 leaks on this coach's page in 5 minutes.</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>media/v2/d15a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>captions/d15a.txt</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>15</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>P15B</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>4 leaks on this coach's page in 5 minutes.</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>media/reels/d15a.mp4</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>captions/d15a.txt</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>16</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>P16A</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>How to answer “Can you reduce the price?”</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>media/reels/d16a.mp4</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>captions/d16a.txt</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>16</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>P16A</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>How to answer “Can you reduce the price?”</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>media/v2/d16a/d16a.pdf</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>captions/d16a.txt</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>16</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>P16A</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>How to answer “Can you reduce the price?”</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>media/reels/d16a.mp4</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>captions/d16a.txt</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>17</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>P17A</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>“How do I make my first sale on my online course?”</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>media/reels/d17b.mp4</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>captions/d17b.txt</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>17</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>P17A</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>“How do I make my first sale on my online course?”</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>media/v2/d17b/d17b.pdf</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>captions/d17b.txt</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>17</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>P17A</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>“How do I make my first sale on my online course?”</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>media/reels/d17b.mp4</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>captions/d17b.txt</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>17</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>P17B</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>If your partner has to book an appointment to see you, your business isn't working. You are.</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>media/v2/p17b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>captions/p17b.txt</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>17</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>P17B</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>If your partner has to book an appointment to see you, your business isn't working. You are.</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>media/reels/p17b.mp4</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>captions/p17b.txt</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>18</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>P18A</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Broke coaches post for likes. Paid coaches post for DMs.</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>media/reels/p18a.mp4</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>captions/p18a.txt</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>18</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>P18B</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Your ad isn't bad. The place it sends people is.</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>media/v2/d19a/d19a.pdf</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>captions/d19a.txt</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>18</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>P18A</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Broke coaches post for likes. Paid coaches post for DMs.</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>media/reels/p18a.mp4</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>captions/p18a.txt</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>18</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>P18B</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Your ad isn't bad. The place it sends people is.</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>media/v2/d19a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>captions/d19a.txt</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>18</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>P18B</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Your ad isn't bad. The place it sends people is.</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>media/reels/d19a.mp4</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>captions/d19a.txt</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>19</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>P19A</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Your bio is a billboard on Third Mainland Bridge.</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>media/reels/d20a.mp4</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>captions/d20a.txt</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>19</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>P19A</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Your bio is a billboard on Third Mainland Bridge.</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>media/v2/d20a/d20a.pdf</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>captions/d20a.txt</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>19</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>P19A</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Your bio is a billboard on Third Mainland Bridge.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>media/reels/d20a.mp4</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>captions/d20a.txt</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>19</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>P19B</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Why I build the page myself.</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>media/v2/d18a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>captions/d18a.txt</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>19</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>P19B</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Why I build the page myself.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>media/reels/d18a.mp4</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>captions/d18a.txt</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>20</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>P20A</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Your family calls it “that your online thing”. Fix that in one sentence.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>media/reels/p20a.mp4</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>captions/p20a.txt</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>20</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>P20B</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>You're not unlucky. You're unmeasured.</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>media/v2/p20b/p20b.pdf</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>captions/p20b.txt</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>20</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>P20A</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Your family calls it “that your online thing”. Fix that in one sentence.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>media/reels/p20a.mp4</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>captions/p20a.txt</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>20</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>P20B</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>You're not unlucky. You're unmeasured.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>media/v2/p20b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>captions/p20b.txt</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>20</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>P20B</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>You're not unlucky. You're unmeasured.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>media/reels/p20b.mp4</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>captions/p20b.txt</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>22</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>P22A</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>If you won't sell your program, someone less skilled will sell theirs to your students.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>media/reels/p22a.mp4</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>captions/p22a.txt</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>22</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>P22B</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Fix these 7 leaks before Black Friday.</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>media/v2/d22a/d22a.pdf</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>captions/d22a.txt</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>22</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>P22A</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>If you won't sell your program, someone less skilled will sell theirs to your students.</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>media/reels/p22a.mp4</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>captions/p22a.txt</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>22</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>P22B</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Fix these 7 leaks before Black Friday.</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>media/v2/d22a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>captions/d22a.txt</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>22</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>P22B</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Fix these 7 leaks before Black Friday.</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>media/reels/d22a.mp4</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>captions/d22a.txt</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>23</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>P23A</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>The market doesn't pay for effort. It pays for clarity.</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>media/reels/p23a.mp4</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>captions/p23a.txt</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>23</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>P23A</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>The market doesn't pay for effort. It pays for clarity.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>media/v2/p23a/p23a.pdf</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>captions/p23a.txt</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>23</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>P23A</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>The market doesn't pay for effort. It pays for clarity.</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>media/reels/p23a.mp4</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>captions/p23a.txt</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>23</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>P23B</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Never fight about money on a bad sales day.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>media/v2/p23b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>captions/p23b.txt</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>23</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>P23B</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Never fight about money on a bad sales day.</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>media/reels/p23b.mp4</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>captions/p23b.txt</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>24</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>P24A</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>What happens when you book a Leak Map.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>media/reels/d23a.mp4</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>captions/d23a.txt</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>24</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>P24A</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>What happens when you book a Leak Map.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>media/v2/d23a/d23a.pdf</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>captions/d23a.txt</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>24</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>P24A</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>What happens when you book a Leak Map.</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>media/reels/d23a.mp4</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>captions/d23a.txt</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>24</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>P24B</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Cost per paying student.</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>media/v2/d22b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>captions/d22b.txt</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>24</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>P24B</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Cost per paying student.</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>media/reels/d22b.mp4</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>captions/d22b.txt</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>25</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>P25A</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Every ignored DM is tuition. You already paid. Collect the lesson.</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>media/reels/p25a.mp4</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>captions/p25a.txt</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>25</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>P25B</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>“I can't afford a marketer.”</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>media/v2/d29b/d29b.pdf</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>captions/d29b.txt</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>25</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>P25A</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Every ignored DM is tuition. You already paid. Collect the lesson.</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>media/reels/p25a.mp4</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>captions/p25a.txt</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>25</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>P25B</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>“I can't afford a marketer.”</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>media/v2/d29b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>captions/d29b.txt</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>25</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>P25B</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>“I can't afford a marketer.”</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>media/reels/d29b.mp4</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>captions/d29b.txt</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>26</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>P26A</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Who is it for? What do they get? Why now?</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>media/reels/d26a.mp4</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>captions/d26a.txt</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>26</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>P26A</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Who is it for? What do they get? Why now?</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>media/v2/d26a/d26a.pdf</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>captions/d26a.txt</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>26</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>P26A</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Who is it for? What do they get? Why now?</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>media/reels/d26a.mp4</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>captions/d26a.txt</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>26</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>P26B</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>The word I never write in health ads.</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>media/v2/d25a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>captions/d25a.txt</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>26</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>P26B</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>The word I never write in health ads.</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>media/reels/d25a.mp4</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>captions/d25a.txt</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>27</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>P27A</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Your spouse thinks online business is “yahoo”. Don't argue. Do this.</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>media/reels/p27a.mp4</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>captions/p27a.txt</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>27</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>P27B</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Your first cohort doesn't need 1,000 followers. It needs 10 real conversations.</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>media/v2/p27b/p27b.pdf</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>captions/p27b.txt</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>27</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>P27A</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Your spouse thinks online business is “yahoo”. Don't argue. Do this.</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>media/reels/p27a.mp4</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>captions/p27a.txt</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>27</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>P27B</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Your first cohort doesn't need 1,000 followers. It needs 10 real conversations.</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>media/v2/p27b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>captions/p27b.txt</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>27</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>P27B</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Your first cohort doesn't need 1,000 followers. It needs 10 real conversations.</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>media/reels/p27b.mp4</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>captions/p27b.txt</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>28</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>P28B</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Black Friday Leak Maps: 5 slots.</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>media/v2/d28b/d28b.pdf</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>captions/d28b.txt</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>28</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>P28B</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Black Friday Leak Maps: 5 slots.</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>media/v2/d28b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>captions/d28b.txt</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>28</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>P28B</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Black Friday Leak Maps: 5 slots.</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>media/reels/d28b.mp4</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>captions/d28b.txt</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>29</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>P29A</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Ready is a feeling. Launch is a date.</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>media/reels/p29a.mp4</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>captions/p29a.txt</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>29</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>P29B</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>How I score a first line out of 50.</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>media/v2/d29a/d29a.pdf</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>captions/d29a.txt</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>29</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>P29A</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Ready is a feeling. Launch is a date.</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>media/reels/p29a.mp4</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>captions/p29a.txt</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>29</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>P29B</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>How I score a first line out of 50.</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>media/v2/d29a/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>captions/d29a.txt</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>29</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>P29B</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>How I score a first line out of 50.</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>media/reels/d29a.mp4</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>captions/d29a.txt</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>30</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Reel (video with music)</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>P30A</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>The 5 leaks on one page.</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>media/reels/d30a.mp4</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>captions/d30a.txt</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>30</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>PDF document (carousel)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>P30A</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>The 5 leaks on one page.</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>media/v2/d30a/d30a.pdf</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>captions/d30a.txt</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>30</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>P30A</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>The 5 leaks on one page.</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>media/reels/d30a.mp4</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>captions/d30a.txt</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>30</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Instagram (auto shares to Facebook)</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Carousel (slides in order)</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>P30B</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Day 30: what's next.</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>media/v2/d30b/01.jpg to last</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>captions/d30b.txt</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Automatic</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>30</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Video with music</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>P30B</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Day 30: what's next.</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>media/reels/d30b.mp4</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>captions/d30b.txt</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Buffer ping: you post it and add a sound</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Approved, not yet in Buffer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L67"/>
+  <autoFilter ref="A1:L138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Free tool: The Hook Scorecard (PDF for Linktree); Instagram posts now go through Buffer pings
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW9n8unhL8LSAM1TzockVG
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1097,7 +1097,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Carousel (slides in order)</t>
+          <t>Reel (video with music)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>media/v2/d04a/01.jpg to last</t>
+          <t>media/reels/d04a.mp4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Carousel (slides in order)</t>
+          <t>Reel (video with music)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>media/v2/d05a/01.jpg to last</t>
+          <t>media/reels/d05a.mp4</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Carousel (slides in order)</t>
+          <t>Reel (video with music)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>media/v2/d06a/01.jpg to last</t>
+          <t>media/reels/d06a.mp4</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Carousel (slides in order)</t>
+          <t>Reel (video with music)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>media/v2/d07a/01.jpg to last</t>
+          <t>media/reels/d07a.mp4</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>Buffer ping: you post it and add a sound</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">

</xml_diff>

<commit_message>
Review PDFs for Days 31 to 60 and the October news posts; schedule refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW9n8unhL8LSAM1TzockVG
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -2422,7 +2422,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schedule: Buffer refill 1 Oct
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW9n8unhL8LSAM1TzockVG
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>In Buffer</t>
+          <t>Posted</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Approved, not yet in Buffer</t>
+          <t>In Buffer</t>
         </is>
       </c>
     </row>

</xml_diff>